<commit_message>
Revert "Merge branch 'master' of https://github.com/sakunamary/artisan"
This reverts commit a18384472c68d6987dd9ab1d38df67b9b54282f4, reversing
changes made to da9d3a301fc435f1aa57b5e1aa000741597bf6c4.
</commit_message>
<xml_diff>
--- a/doc/help_dialogs/Input_files/eventbuttons.xlsx
+++ b/doc/help_dialogs/Input_files/eventbuttons.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="Buttons" sheetId="1" state="visible" r:id="rId3"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="424" uniqueCount="379">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="424" uniqueCount="378">
   <si>
     <t xml:space="preserve">EVENT CUSTOM BUTTONS</t>
   </si>
@@ -299,9 +299,6 @@
   </si>
   <si>
     <t xml:space="preserve">FILL</t>
-  </si>
-  <si>
-    <t xml:space="preserve">\\D</t>
   </si>
   <si>
     <t xml:space="preserve">DISCHARGE</t>
@@ -745,22 +742,22 @@
     <t xml:space="preserve">PHIDGET PWM Output: turn &lt;channel&gt; on for &lt;millis&gt; milliseconds</t>
   </si>
   <si>
-    <t xml:space="preserve">outhub(&lt;port&gt;,&lt;value&gt;[,&lt;sn&gt;])</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PHIDGET HUB PWM Output ON port &lt;port&gt; to  &lt;value&gt; in [0-100]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">togglehub(&lt;port&gt;[,&lt;sn&gt;])</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PHIDGET HUB PWM Output: toggles &lt;port&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">pulsehub(&lt;port&gt;,&lt;millis&gt;[,&lt;sn&gt;])</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PHIDGET HUB PWM Output:  turn &lt;port&gt; ON for &lt;millis&gt; milliseconds</t>
+    <t xml:space="preserve">outhub(&lt;channel&gt;,&lt;value&gt;[,&lt;sn&gt;])</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PHIDGET HUB PWM Output: &lt;value&gt; in [0-100]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">togglehub(&lt;channel&gt;[,&lt;sn&gt;])</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PHIDGET HUB PWM Output: toggles &lt;channel&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pulsehub(&lt;channel&gt;,&lt;millis&gt;[,&lt;sn&gt;])</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PHIDGET HUB PWM Output:  turn &lt;channel&gt; on for &lt;millis&gt; milliseconds</t>
   </si>
   <si>
     <t xml:space="preserve">enabled(c,b[,sn])</t>
@@ -1851,74 +1848,74 @@
     </row>
     <row r="28" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="B28" s="1" t="s">
         <v>92</v>
-      </c>
-      <c r="B28" s="1" t="s">
-        <v>93</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="B29" s="1" t="s">
         <v>94</v>
-      </c>
-      <c r="B29" s="1" t="s">
-        <v>95</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="B30" s="1" t="s">
         <v>96</v>
-      </c>
-      <c r="B30" s="1" t="s">
-        <v>97</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="B31" s="1" t="s">
         <v>98</v>
-      </c>
-      <c r="B31" s="1" t="s">
-        <v>99</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="B32" s="1" t="s">
         <v>100</v>
-      </c>
-      <c r="B32" s="1" t="s">
-        <v>101</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="B33" s="1" t="s">
         <v>102</v>
-      </c>
-      <c r="B33" s="1" t="s">
-        <v>103</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="B34" s="1" t="s">
         <v>104</v>
-      </c>
-      <c r="B34" s="1" t="s">
-        <v>105</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="B35" s="1" t="s">
         <v>106</v>
-      </c>
-      <c r="B35" s="1" t="s">
-        <v>107</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="B36" s="1" t="s">
         <v>108</v>
-      </c>
-      <c r="B36" s="1" t="s">
-        <v>109</v>
       </c>
     </row>
   </sheetData>
@@ -1940,44 +1937,44 @@
   <dimension ref="A1:C153"/>
   <sheetFormatPr defaultColWidth="9.265625" defaultRowHeight="14.5" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="26.74"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="112.84"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="54.54"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="100.36"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1985,7 +1982,7 @@
         <v>12</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>3</v>
@@ -1993,1201 +1990,1201 @@
     </row>
     <row r="9" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="B9" s="1" t="s">
         <v>118</v>
-      </c>
-      <c r="B9" s="1" t="s">
-        <v>119</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="B10" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="B10" s="1" t="s">
+      <c r="C10" s="1" t="s">
         <v>121</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="B11" s="1" t="s">
         <v>123</v>
       </c>
-      <c r="B11" s="1" t="s">
+      <c r="C11" s="1" t="s">
         <v>124</v>
-      </c>
-      <c r="C11" s="1" t="s">
-        <v>125</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="B12" s="3" t="s">
         <v>126</v>
       </c>
-      <c r="B12" s="3" t="s">
+      <c r="C12" s="1" t="s">
         <v>127</v>
-      </c>
-      <c r="C12" s="1" t="s">
-        <v>128</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="C13" s="1" t="s">
         <v>129</v>
-      </c>
-      <c r="C13" s="1" t="s">
-        <v>130</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="C14" s="1" t="s">
         <v>131</v>
-      </c>
-      <c r="C14" s="1" t="s">
-        <v>132</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="C15" s="1" t="s">
         <v>133</v>
-      </c>
-      <c r="C15" s="1" t="s">
-        <v>134</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="C16" s="1" t="s">
         <v>135</v>
-      </c>
-      <c r="C16" s="1" t="s">
-        <v>136</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="C17" s="1" t="s">
         <v>137</v>
-      </c>
-      <c r="C17" s="1" t="s">
-        <v>138</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="3" t="s">
+        <v>138</v>
+      </c>
+      <c r="C18" s="1" t="s">
         <v>139</v>
-      </c>
-      <c r="C18" s="1" t="s">
-        <v>140</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="3" t="s">
+        <v>140</v>
+      </c>
+      <c r="C19" s="1" t="s">
         <v>141</v>
-      </c>
-      <c r="C19" s="1" t="s">
-        <v>142</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="C20" s="1" t="s">
         <v>143</v>
-      </c>
-      <c r="C20" s="1" t="s">
-        <v>144</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="3" t="s">
+        <v>144</v>
+      </c>
+      <c r="C21" s="1" t="s">
         <v>145</v>
-      </c>
-      <c r="C21" s="1" t="s">
-        <v>146</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="3" t="s">
+        <v>146</v>
+      </c>
+      <c r="C22" s="1" t="s">
         <v>147</v>
-      </c>
-      <c r="C22" s="1" t="s">
-        <v>148</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B23" s="3" t="s">
+        <v>148</v>
+      </c>
+      <c r="C23" s="1" t="s">
         <v>149</v>
-      </c>
-      <c r="C23" s="1" t="s">
-        <v>150</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B24" s="3" t="s">
+        <v>150</v>
+      </c>
+      <c r="C24" s="1" t="s">
         <v>151</v>
-      </c>
-      <c r="C24" s="1" t="s">
-        <v>152</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="C25" s="1" t="s">
         <v>153</v>
-      </c>
-      <c r="C25" s="1" t="s">
-        <v>154</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B26" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="C26" s="1" t="s">
         <v>155</v>
-      </c>
-      <c r="C26" s="1" t="s">
-        <v>156</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="3" t="s">
+        <v>156</v>
+      </c>
+      <c r="C27" s="1" t="s">
         <v>157</v>
-      </c>
-      <c r="C27" s="1" t="s">
-        <v>158</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B28" s="3" t="s">
+        <v>158</v>
+      </c>
+      <c r="C28" s="1" t="s">
         <v>159</v>
-      </c>
-      <c r="C28" s="1" t="s">
-        <v>160</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B29" s="3" t="s">
+        <v>160</v>
+      </c>
+      <c r="C29" s="1" t="s">
         <v>161</v>
-      </c>
-      <c r="C29" s="1" t="s">
-        <v>162</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B30" s="3" t="s">
+        <v>162</v>
+      </c>
+      <c r="C30" s="1" t="s">
         <v>163</v>
-      </c>
-      <c r="C30" s="1" t="s">
-        <v>164</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B31" s="3" t="s">
+        <v>164</v>
+      </c>
+      <c r="C31" s="1" t="s">
         <v>165</v>
-      </c>
-      <c r="C31" s="1" t="s">
-        <v>166</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B32" s="3" t="s">
+        <v>166</v>
+      </c>
+      <c r="C32" s="1" t="s">
         <v>167</v>
-      </c>
-      <c r="C32" s="1" t="s">
-        <v>168</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B33" s="3" t="s">
+        <v>168</v>
+      </c>
+      <c r="C33" s="1" t="s">
         <v>169</v>
-      </c>
-      <c r="C33" s="1" t="s">
-        <v>170</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="1" t="s">
+        <v>170</v>
+      </c>
+      <c r="B34" s="1" t="s">
         <v>171</v>
-      </c>
-      <c r="B34" s="1" t="s">
-        <v>172</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="1" t="s">
+        <v>172</v>
+      </c>
+      <c r="B35" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="C35" s="1" t="s">
         <v>173</v>
-      </c>
-      <c r="B35" s="3" t="s">
-        <v>127</v>
-      </c>
-      <c r="C35" s="1" t="s">
-        <v>174</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B36" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="C36" s="1" t="s">
         <v>129</v>
-      </c>
-      <c r="C36" s="1" t="s">
-        <v>130</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B37" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="C37" s="1" t="s">
         <v>175</v>
-      </c>
-      <c r="C37" s="1" t="s">
-        <v>176</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B38" s="3" t="s">
+        <v>176</v>
+      </c>
+      <c r="C38" s="1" t="s">
         <v>177</v>
-      </c>
-      <c r="C38" s="1" t="s">
-        <v>178</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B39" s="3" t="s">
+        <v>178</v>
+      </c>
+      <c r="C39" s="1" t="s">
         <v>179</v>
-      </c>
-      <c r="C39" s="1" t="s">
-        <v>180</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B40" s="3" t="s">
+        <v>180</v>
+      </c>
+      <c r="C40" s="1" t="s">
         <v>181</v>
-      </c>
-      <c r="C40" s="1" t="s">
-        <v>182</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B41" s="3" t="s">
+        <v>182</v>
+      </c>
+      <c r="C41" s="1" t="s">
         <v>183</v>
-      </c>
-      <c r="C41" s="1" t="s">
-        <v>184</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B42" s="3" t="s">
+        <v>184</v>
+      </c>
+      <c r="C42" s="1" t="s">
         <v>185</v>
-      </c>
-      <c r="C42" s="1" t="s">
-        <v>186</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B43" s="3" t="s">
+        <v>186</v>
+      </c>
+      <c r="C43" s="1" t="s">
         <v>187</v>
-      </c>
-      <c r="C43" s="1" t="s">
-        <v>188</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B44" s="3" t="s">
+        <v>188</v>
+      </c>
+      <c r="C44" s="1" t="s">
         <v>189</v>
-      </c>
-      <c r="C44" s="1" t="s">
-        <v>190</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B45" s="3" t="s">
+        <v>190</v>
+      </c>
+      <c r="C45" s="1" t="s">
         <v>191</v>
-      </c>
-      <c r="C45" s="1" t="s">
-        <v>192</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B46" s="3" t="s">
+        <v>192</v>
+      </c>
+      <c r="C46" s="1" t="s">
         <v>193</v>
-      </c>
-      <c r="C46" s="1" t="s">
-        <v>194</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B47" s="3" t="s">
+        <v>194</v>
+      </c>
+      <c r="C47" s="1" t="s">
         <v>195</v>
-      </c>
-      <c r="C47" s="1" t="s">
-        <v>196</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B48" s="3" t="s">
+        <v>196</v>
+      </c>
+      <c r="C48" s="1" t="s">
         <v>197</v>
-      </c>
-      <c r="C48" s="1" t="s">
-        <v>198</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B49" s="3" t="s">
+        <v>198</v>
+      </c>
+      <c r="C49" s="1" t="s">
         <v>199</v>
-      </c>
-      <c r="C49" s="1" t="s">
-        <v>200</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B50" s="3" t="s">
+        <v>200</v>
+      </c>
+      <c r="C50" s="1" t="s">
         <v>201</v>
-      </c>
-      <c r="C50" s="1" t="s">
-        <v>202</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B51" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="C51" s="1" t="s">
         <v>203</v>
-      </c>
-      <c r="C51" s="1" t="s">
-        <v>204</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B52" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="C52" s="1" t="s">
         <v>133</v>
-      </c>
-      <c r="C52" s="1" t="s">
-        <v>134</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B53" s="3" t="s">
+        <v>204</v>
+      </c>
+      <c r="C53" s="1" t="s">
         <v>205</v>
-      </c>
-      <c r="C53" s="1" t="s">
-        <v>206</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B54" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="C54" s="1" t="s">
         <v>137</v>
-      </c>
-      <c r="C54" s="1" t="s">
-        <v>138</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B55" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="C55" s="1" t="s">
         <v>131</v>
-      </c>
-      <c r="C55" s="1" t="s">
-        <v>132</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B56" s="3" t="s">
+        <v>206</v>
+      </c>
+      <c r="C56" s="1" t="s">
         <v>207</v>
-      </c>
-      <c r="C56" s="1" t="s">
-        <v>208</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B57" s="3" t="s">
+        <v>208</v>
+      </c>
+      <c r="C57" s="1" t="s">
         <v>209</v>
-      </c>
-      <c r="C57" s="1" t="s">
-        <v>210</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="1" t="s">
+        <v>210</v>
+      </c>
+      <c r="C58" s="1" t="s">
         <v>211</v>
-      </c>
-      <c r="C58" s="1" t="s">
-        <v>212</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="1" t="s">
+        <v>212</v>
+      </c>
+      <c r="C59" s="1" t="s">
         <v>213</v>
-      </c>
-      <c r="C59" s="1" t="s">
-        <v>214</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="1" t="s">
+        <v>214</v>
+      </c>
+      <c r="B60" s="4" t="s">
         <v>215</v>
       </c>
-      <c r="B60" s="4" t="s">
+      <c r="C60" s="1" t="s">
         <v>216</v>
-      </c>
-      <c r="C60" s="1" t="s">
-        <v>217</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="1" t="s">
+        <v>217</v>
+      </c>
+      <c r="B61" s="3" t="s">
         <v>218</v>
       </c>
-      <c r="B61" s="3" t="s">
+      <c r="C61" s="1" t="s">
         <v>219</v>
-      </c>
-      <c r="C61" s="1" t="s">
-        <v>220</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="1" t="s">
+        <v>220</v>
+      </c>
+      <c r="B62" s="3" t="s">
         <v>221</v>
-      </c>
-      <c r="B62" s="3" t="s">
-        <v>222</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="1" t="s">
+        <v>222</v>
+      </c>
+      <c r="B63" s="3" t="s">
         <v>223</v>
       </c>
-      <c r="B63" s="3" t="s">
+      <c r="C63" s="1" t="s">
         <v>224</v>
-      </c>
-      <c r="C63" s="1" t="s">
-        <v>225</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B64" s="3" t="s">
+        <v>225</v>
+      </c>
+      <c r="C64" s="1" t="s">
         <v>226</v>
-      </c>
-      <c r="C64" s="1" t="s">
-        <v>227</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B65" s="3" t="s">
+        <v>227</v>
+      </c>
+      <c r="C65" s="1" t="s">
         <v>228</v>
-      </c>
-      <c r="C65" s="1" t="s">
-        <v>229</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B66" s="3" t="s">
+        <v>229</v>
+      </c>
+      <c r="C66" s="1" t="s">
         <v>230</v>
-      </c>
-      <c r="C66" s="1" t="s">
-        <v>231</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B67" s="3" t="s">
+        <v>231</v>
+      </c>
+      <c r="C67" s="1" t="s">
         <v>232</v>
-      </c>
-      <c r="C67" s="1" t="s">
-        <v>233</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B68" s="3" t="s">
+        <v>233</v>
+      </c>
+      <c r="C68" s="1" t="s">
         <v>234</v>
-      </c>
-      <c r="C68" s="1" t="s">
-        <v>235</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B69" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="C69" s="1" t="s">
         <v>236</v>
-      </c>
-      <c r="C69" s="1" t="s">
-        <v>237</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B70" s="3" t="s">
+        <v>237</v>
+      </c>
+      <c r="C70" s="1" t="s">
         <v>238</v>
-      </c>
-      <c r="C70" s="1" t="s">
-        <v>239</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B71" s="3" t="s">
+        <v>239</v>
+      </c>
+      <c r="C71" s="1" t="s">
         <v>240</v>
-      </c>
-      <c r="C71" s="1" t="s">
-        <v>241</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B72" s="3" t="s">
+        <v>241</v>
+      </c>
+      <c r="C72" s="1" t="s">
         <v>242</v>
-      </c>
-      <c r="C72" s="1" t="s">
-        <v>243</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="1" t="s">
+        <v>243</v>
+      </c>
+      <c r="B73" s="3" t="s">
         <v>244</v>
       </c>
-      <c r="B73" s="3" t="s">
+      <c r="C73" s="1" t="s">
         <v>245</v>
-      </c>
-      <c r="C73" s="1" t="s">
-        <v>246</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B74" s="3" t="s">
+        <v>246</v>
+      </c>
+      <c r="C74" s="1" t="s">
         <v>247</v>
-      </c>
-      <c r="C74" s="1" t="s">
-        <v>248</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B75" s="3" t="s">
+        <v>248</v>
+      </c>
+      <c r="C75" s="1" t="s">
         <v>249</v>
-      </c>
-      <c r="C75" s="1" t="s">
-        <v>250</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B76" s="3" t="s">
+        <v>250</v>
+      </c>
+      <c r="C76" s="1" t="s">
         <v>251</v>
-      </c>
-      <c r="C76" s="1" t="s">
-        <v>252</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B77" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="C77" s="1" t="s">
         <v>131</v>
-      </c>
-      <c r="C77" s="1" t="s">
-        <v>132</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="1" t="s">
+        <v>252</v>
+      </c>
+      <c r="B78" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="C78" s="1" t="s">
         <v>253</v>
-      </c>
-      <c r="B78" s="3" t="s">
-        <v>127</v>
-      </c>
-      <c r="C78" s="1" t="s">
-        <v>254</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B79" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="C79" s="1" t="s">
         <v>129</v>
-      </c>
-      <c r="C79" s="1" t="s">
-        <v>130</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B80" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="C80" s="1" t="s">
         <v>131</v>
-      </c>
-      <c r="C80" s="1" t="s">
-        <v>132</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B81" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="C81" s="1" t="s">
         <v>133</v>
-      </c>
-      <c r="C81" s="1" t="s">
-        <v>134</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B82" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="C82" s="1" t="s">
         <v>135</v>
-      </c>
-      <c r="C82" s="1" t="s">
-        <v>136</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B83" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="C83" s="1" t="s">
         <v>137</v>
-      </c>
-      <c r="C83" s="1" t="s">
-        <v>138</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B84" s="3" t="s">
+        <v>254</v>
+      </c>
+      <c r="C84" s="1" t="s">
         <v>255</v>
-      </c>
-      <c r="C84" s="1" t="s">
-        <v>256</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B85" s="3" t="s">
+        <v>256</v>
+      </c>
+      <c r="C85" s="1" t="s">
         <v>257</v>
-      </c>
-      <c r="C85" s="1" t="s">
-        <v>258</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B86" s="3" t="s">
+        <v>258</v>
+      </c>
+      <c r="C86" s="1" t="s">
         <v>259</v>
-      </c>
-      <c r="C86" s="1" t="s">
-        <v>260</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B87" s="3" t="s">
+        <v>260</v>
+      </c>
+      <c r="C87" s="1" t="s">
         <v>261</v>
-      </c>
-      <c r="C87" s="1" t="s">
-        <v>262</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B88" s="3" t="s">
+        <v>262</v>
+      </c>
+      <c r="C88" s="1" t="s">
         <v>263</v>
-      </c>
-      <c r="C88" s="1" t="s">
-        <v>264</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B89" s="3" t="s">
+        <v>264</v>
+      </c>
+      <c r="C89" s="1" t="s">
         <v>265</v>
-      </c>
-      <c r="C89" s="1" t="s">
-        <v>266</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B90" s="3" t="s">
+        <v>266</v>
+      </c>
+      <c r="C90" s="1" t="s">
         <v>267</v>
-      </c>
-      <c r="C90" s="1" t="s">
-        <v>268</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A91" s="1" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="C91" s="1" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A92" s="1" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="C92" s="1" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A93" s="1" t="s">
+        <v>270</v>
+      </c>
+      <c r="C93" s="1" t="s">
         <v>271</v>
-      </c>
-      <c r="C93" s="1" t="s">
-        <v>272</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A94" s="1" t="s">
+        <v>272</v>
+      </c>
+      <c r="B94" s="3" t="s">
         <v>273</v>
       </c>
-      <c r="B94" s="3" t="s">
+      <c r="C94" s="1" t="s">
         <v>274</v>
-      </c>
-      <c r="C94" s="1" t="s">
-        <v>275</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="1" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="B95" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="C95" s="1" t="s">
         <v>129</v>
-      </c>
-      <c r="C95" s="1" t="s">
-        <v>130</v>
       </c>
     </row>
     <row r="96" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B96" s="3" t="s">
+        <v>276</v>
+      </c>
+      <c r="C96" s="1" t="s">
         <v>277</v>
-      </c>
-      <c r="C96" s="1" t="s">
-        <v>278</v>
       </c>
     </row>
     <row r="97" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B97" s="3" t="s">
+        <v>278</v>
+      </c>
+      <c r="C97" s="1" t="s">
         <v>279</v>
-      </c>
-      <c r="C97" s="1" t="s">
-        <v>280</v>
       </c>
     </row>
     <row r="98" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B98" s="3" t="s">
+        <v>280</v>
+      </c>
+      <c r="C98" s="1" t="s">
         <v>281</v>
-      </c>
-      <c r="C98" s="1" t="s">
-        <v>282</v>
       </c>
     </row>
     <row r="99" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B99" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="C99" s="1" t="s">
         <v>131</v>
-      </c>
-      <c r="C99" s="1" t="s">
-        <v>132</v>
       </c>
     </row>
     <row r="100" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B100" s="3" t="s">
+        <v>282</v>
+      </c>
+      <c r="C100" s="1" t="s">
         <v>283</v>
-      </c>
-      <c r="C100" s="1" t="s">
-        <v>284</v>
       </c>
     </row>
     <row r="101" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B101" s="3" t="s">
+        <v>284</v>
+      </c>
+      <c r="C101" s="1" t="s">
         <v>285</v>
-      </c>
-      <c r="C101" s="1" t="s">
-        <v>286</v>
       </c>
     </row>
     <row r="102" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B102" s="3" t="s">
+        <v>286</v>
+      </c>
+      <c r="C102" s="1" t="s">
         <v>287</v>
-      </c>
-      <c r="C102" s="1" t="s">
-        <v>288</v>
       </c>
     </row>
     <row r="103" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B103" s="3" t="s">
+        <v>288</v>
+      </c>
+      <c r="C103" s="1" t="s">
         <v>289</v>
-      </c>
-      <c r="C103" s="1" t="s">
-        <v>290</v>
       </c>
     </row>
     <row r="104" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B104" s="3" t="s">
+        <v>290</v>
+      </c>
+      <c r="C104" s="1" t="s">
         <v>291</v>
-      </c>
-      <c r="C104" s="1" t="s">
-        <v>292</v>
       </c>
     </row>
     <row r="105" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B105" s="3" t="s">
+        <v>292</v>
+      </c>
+      <c r="C105" s="1" t="s">
         <v>293</v>
-      </c>
-      <c r="C105" s="1" t="s">
-        <v>294</v>
       </c>
     </row>
     <row r="106" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B106" s="3" t="s">
+        <v>294</v>
+      </c>
+      <c r="C106" s="1" t="s">
         <v>295</v>
-      </c>
-      <c r="C106" s="1" t="s">
-        <v>296</v>
       </c>
     </row>
     <row r="107" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B107" s="3" t="s">
+        <v>296</v>
+      </c>
+      <c r="C107" s="1" t="s">
         <v>297</v>
-      </c>
-      <c r="C107" s="1" t="s">
-        <v>298</v>
       </c>
     </row>
     <row r="108" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B108" s="3" t="s">
+        <v>298</v>
+      </c>
+      <c r="C108" s="1" t="s">
         <v>299</v>
-      </c>
-      <c r="C108" s="1" t="s">
-        <v>300</v>
       </c>
     </row>
     <row r="109" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B109" s="3" t="s">
+        <v>300</v>
+      </c>
+      <c r="C109" s="1" t="s">
         <v>301</v>
-      </c>
-      <c r="C109" s="1" t="s">
-        <v>302</v>
       </c>
     </row>
     <row r="110" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B110" s="3" t="s">
+        <v>302</v>
+      </c>
+      <c r="C110" s="1" t="s">
         <v>303</v>
-      </c>
-      <c r="C110" s="1" t="s">
-        <v>304</v>
       </c>
     </row>
     <row r="111" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B111" s="3" t="s">
+        <v>304</v>
+      </c>
+      <c r="C111" s="1" t="s">
         <v>305</v>
-      </c>
-      <c r="C111" s="1" t="s">
-        <v>306</v>
       </c>
     </row>
     <row r="112" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B112" s="3" t="s">
+        <v>306</v>
+      </c>
+      <c r="C112" s="1" t="s">
         <v>307</v>
-      </c>
-      <c r="C112" s="1" t="s">
-        <v>308</v>
       </c>
     </row>
     <row r="113" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B113" s="3" t="s">
+        <v>308</v>
+      </c>
+      <c r="C113" s="1" t="s">
         <v>309</v>
-      </c>
-      <c r="C113" s="1" t="s">
-        <v>310</v>
       </c>
     </row>
     <row r="114" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B114" s="3" t="s">
+        <v>310</v>
+      </c>
+      <c r="C114" s="1" t="s">
         <v>311</v>
-      </c>
-      <c r="C114" s="1" t="s">
-        <v>312</v>
       </c>
     </row>
     <row r="115" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B115" s="3" t="s">
+        <v>312</v>
+      </c>
+      <c r="C115" s="1" t="s">
         <v>313</v>
-      </c>
-      <c r="C115" s="1" t="s">
-        <v>314</v>
       </c>
     </row>
     <row r="116" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B116" s="3" t="s">
+        <v>314</v>
+      </c>
+      <c r="C116" s="1" t="s">
         <v>315</v>
-      </c>
-      <c r="C116" s="1" t="s">
-        <v>316</v>
       </c>
     </row>
     <row r="117" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B117" s="3" t="s">
+        <v>316</v>
+      </c>
+      <c r="C117" s="1" t="s">
         <v>317</v>
-      </c>
-      <c r="C117" s="1" t="s">
-        <v>318</v>
       </c>
     </row>
     <row r="118" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B118" s="3" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C118" s="1" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
     </row>
     <row r="119" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B119" s="3" t="s">
+        <v>319</v>
+      </c>
+      <c r="C119" s="1" t="s">
         <v>320</v>
-      </c>
-      <c r="C119" s="1" t="s">
-        <v>321</v>
       </c>
     </row>
     <row r="120" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B120" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="C120" s="1" t="s">
         <v>137</v>
-      </c>
-      <c r="C120" s="1" t="s">
-        <v>138</v>
       </c>
     </row>
     <row r="121" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B121" s="3" t="s">
+        <v>321</v>
+      </c>
+      <c r="C121" s="1" t="s">
         <v>322</v>
-      </c>
-      <c r="C121" s="1" t="s">
-        <v>323</v>
       </c>
     </row>
     <row r="122" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B122" s="3" t="s">
+        <v>323</v>
+      </c>
+      <c r="C122" s="1" t="s">
         <v>324</v>
-      </c>
-      <c r="C122" s="1" t="s">
-        <v>325</v>
       </c>
     </row>
     <row r="123" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B123" s="3" t="s">
+        <v>325</v>
+      </c>
+      <c r="C123" s="1" t="s">
         <v>326</v>
-      </c>
-      <c r="C123" s="1" t="s">
-        <v>327</v>
       </c>
     </row>
     <row r="124" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B124" s="3" t="s">
+        <v>327</v>
+      </c>
+      <c r="C124" s="1" t="s">
         <v>328</v>
-      </c>
-      <c r="C124" s="1" t="s">
-        <v>329</v>
       </c>
     </row>
     <row r="125" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B125" s="3" t="s">
+        <v>329</v>
+      </c>
+      <c r="C125" s="1" t="s">
         <v>330</v>
-      </c>
-      <c r="C125" s="1" t="s">
-        <v>331</v>
       </c>
     </row>
     <row r="126" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B126" s="3" t="s">
+        <v>331</v>
+      </c>
+      <c r="C126" s="1" t="s">
         <v>332</v>
-      </c>
-      <c r="C126" s="1" t="s">
-        <v>333</v>
       </c>
     </row>
     <row r="127" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B127" s="3" t="s">
+        <v>333</v>
+      </c>
+      <c r="C127" s="1" t="s">
         <v>334</v>
-      </c>
-      <c r="C127" s="1" t="s">
-        <v>335</v>
       </c>
     </row>
     <row r="128" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B128" s="3" t="s">
+        <v>335</v>
+      </c>
+      <c r="C128" s="1" t="s">
         <v>336</v>
-      </c>
-      <c r="C128" s="1" t="s">
-        <v>337</v>
       </c>
     </row>
     <row r="129" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B129" s="3" t="s">
+        <v>337</v>
+      </c>
+      <c r="C129" s="1" t="s">
         <v>338</v>
-      </c>
-      <c r="C129" s="1" t="s">
-        <v>339</v>
       </c>
     </row>
     <row r="130" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B130" s="3" t="s">
+        <v>339</v>
+      </c>
+      <c r="C130" s="1" t="s">
         <v>340</v>
-      </c>
-      <c r="C130" s="1" t="s">
-        <v>341</v>
       </c>
     </row>
     <row r="131" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B131" s="3" t="s">
+        <v>341</v>
+      </c>
+      <c r="C131" s="1" t="s">
         <v>342</v>
-      </c>
-      <c r="C131" s="1" t="s">
-        <v>343</v>
       </c>
     </row>
     <row r="132" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B132" s="3" t="s">
+        <v>343</v>
+      </c>
+      <c r="C132" s="1" t="s">
         <v>344</v>
-      </c>
-      <c r="C132" s="1" t="s">
-        <v>345</v>
       </c>
     </row>
     <row r="133" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B133" s="3" t="s">
+        <v>345</v>
+      </c>
+      <c r="C133" s="1" t="s">
         <v>346</v>
-      </c>
-      <c r="C133" s="1" t="s">
-        <v>347</v>
       </c>
     </row>
     <row r="134" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B134" s="3" t="s">
+        <v>347</v>
+      </c>
+      <c r="C134" s="1" t="s">
         <v>348</v>
-      </c>
-      <c r="C134" s="1" t="s">
-        <v>349</v>
       </c>
     </row>
     <row r="135" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A135" s="1" t="s">
+        <v>349</v>
+      </c>
+      <c r="B135" s="3" t="s">
         <v>350</v>
       </c>
-      <c r="B135" s="3" t="s">
+      <c r="C135" s="1" t="s">
         <v>351</v>
-      </c>
-      <c r="C135" s="1" t="s">
-        <v>352</v>
       </c>
     </row>
     <row r="136" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B136" s="3" t="s">
+        <v>352</v>
+      </c>
+      <c r="C136" s="1" t="s">
         <v>353</v>
-      </c>
-      <c r="C136" s="1" t="s">
-        <v>354</v>
       </c>
     </row>
     <row r="137" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B137" s="3" t="s">
+        <v>354</v>
+      </c>
+      <c r="C137" s="1" t="s">
         <v>355</v>
-      </c>
-      <c r="C137" s="1" t="s">
-        <v>356</v>
       </c>
     </row>
     <row r="138" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B138" s="3" t="s">
+        <v>356</v>
+      </c>
+      <c r="C138" s="1" t="s">
         <v>357</v>
-      </c>
-      <c r="C138" s="1" t="s">
-        <v>358</v>
       </c>
     </row>
     <row r="139" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B139" s="3" t="s">
+        <v>358</v>
+      </c>
+      <c r="C139" s="1" t="s">
         <v>359</v>
-      </c>
-      <c r="C139" s="1" t="s">
-        <v>360</v>
       </c>
     </row>
     <row r="140" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B140" s="3" t="s">
+        <v>360</v>
+      </c>
+      <c r="C140" s="1" t="s">
         <v>361</v>
-      </c>
-      <c r="C140" s="1" t="s">
-        <v>362</v>
       </c>
     </row>
     <row r="141" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B141" s="3" t="s">
+        <v>362</v>
+      </c>
+      <c r="C141" s="1" t="s">
         <v>363</v>
-      </c>
-      <c r="C141" s="1" t="s">
-        <v>364</v>
       </c>
     </row>
     <row r="142" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B142" s="3" t="s">
+        <v>364</v>
+      </c>
+      <c r="C142" s="1" t="s">
         <v>365</v>
-      </c>
-      <c r="C142" s="1" t="s">
-        <v>366</v>
       </c>
     </row>
     <row r="143" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B143" s="3" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="C143" s="1" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
     </row>
     <row r="144" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B144" s="3" t="s">
+        <v>367</v>
+      </c>
+      <c r="C144" s="1" t="s">
         <v>368</v>
-      </c>
-      <c r="C144" s="1" t="s">
-        <v>369</v>
       </c>
     </row>
     <row r="145" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B145" s="3" t="s">
+        <v>369</v>
+      </c>
+      <c r="C145" s="1" t="s">
         <v>370</v>
-      </c>
-      <c r="C145" s="1" t="s">
-        <v>371</v>
       </c>
     </row>
     <row r="146" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B146" s="3" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="C146" s="1" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="147" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A147" s="1" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="B147" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="C147" s="1" t="s">
         <v>129</v>
-      </c>
-      <c r="C147" s="1" t="s">
-        <v>130</v>
       </c>
     </row>
     <row r="148" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B148" s="3" t="s">
+        <v>373</v>
+      </c>
+      <c r="C148" s="1" t="s">
         <v>374</v>
-      </c>
-      <c r="C148" s="1" t="s">
-        <v>375</v>
       </c>
     </row>
     <row r="149" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B149" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="C149" s="1" t="s">
         <v>131</v>
-      </c>
-      <c r="C149" s="1" t="s">
-        <v>132</v>
       </c>
     </row>
     <row r="150" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B150" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="C150" s="1" t="s">
         <v>133</v>
-      </c>
-      <c r="C150" s="1" t="s">
-        <v>134</v>
       </c>
     </row>
     <row r="151" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B151" s="3" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="C151" s="1" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
     </row>
     <row r="152" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B152" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="C152" s="1" t="s">
         <v>137</v>
-      </c>
-      <c r="C152" s="1" t="s">
-        <v>138</v>
       </c>
     </row>
     <row r="153" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B153" s="3" t="s">
+        <v>376</v>
+      </c>
+      <c r="C153" s="1" t="s">
         <v>377</v>
-      </c>
-      <c r="C153" s="1" t="s">
-        <v>378</v>
       </c>
     </row>
   </sheetData>

</xml_diff>